<commit_message>
refactor: english headers + expected results in XLSX
</commit_message>
<xml_diff>
--- a/projects/akademi-competition/test-cases.xlsx
+++ b/projects/akademi-competition/test-cases.xlsx
@@ -479,12 +479,13 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Modul</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -494,12 +495,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -664,7 +665,7 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
@@ -672,47 +673,47 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>TC ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Modul</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Fitur</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Skenario</t>
+          <t>Scenario</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Prekondisi</t>
+          <t>Precondition</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Langkah</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Hasil Diharapkan</t>
+          <t>Expected Result</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Tipe</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Prioritas</t>
+          <t>Priority</t>
         </is>
       </c>
     </row>
@@ -734,28 +735,28 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Melihat feed artikel (For You tab)</t>
+          <t>View article feed (For You tab)</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Login, punya artikel published</t>
+          <t>Logged in, articles exist in DB</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1. Buka /user/social-forum
-2. Tab For You aktif</t>
+          <t>1. Open /user/social-forum
+2. For You tab is active</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Artikel tampil dalam cards, infinite scroll</t>
+          <t>Article cards displayed with infinite scroll</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -782,28 +783,28 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Search artikel</t>
+          <t>Search articles</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Ada artikel di database</t>
+          <t>Articles exist in DB</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>1. Buka Social Forum
-2. Ketik keyword di search bar</t>
+          <t>1. Open Social Forum
+2. Type keyword in search bar</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Artikel sesuai keyword tampil</t>
+          <t>Matching articles displayed</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -830,28 +831,28 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Filter artikel by tag</t>
+          <t>Filter articles by tag</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Ada tag &amp; artikel dengan tag</t>
+          <t>Tags and tagged articles exist</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>1. Klik filter tag
-2. Pilih 1+ tag</t>
+          <t>1. Click filter button
+2. Select 1+ tags</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Feed terfilter sesuai tag dipilih</t>
+          <t>Feed filtered by selected tags</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -883,22 +884,22 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Ada artikel dengan interaksi</t>
+          <t>Articles with interactions exist</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Scroll ke trending sidebar</t>
+          <t>Scroll to trending sidebar</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Trending articles tampil</t>
+          <t>Trending articles displayed</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -925,33 +926,33 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Membuat artikel baru</t>
+          <t>Create a new article</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Login sebagai user</t>
+          <t>Logged in as user</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1. Klik 'Buat Artikel'
-2. Isi title
-3. Isi body (rich text)
+          <t>1. Click 'Create Article'
+2. Fill title
+3. Fill body (rich text)
 4. Upload cover image
-5. Pilih tag
+5. Select tags
 6. Set visibility
-7. Klik Publish</t>
+7. Click Publish</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Artikel sukses dibuat, muncul di feed</t>
+          <t>Article created successfully, appears in feed</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -978,28 +979,28 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Membuat artikel tanpa cover image</t>
+          <t>Create article without cover image</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>1. Isi semua field kecuali cover
-2. Klik Publish</t>
+          <t>1. Fill all fields except cover
+2. Click Publish</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Validasi: cover image required</t>
+          <t>Validation: cover image is required</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1026,30 +1027,30 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Membuat artikel dengan judul kosong</t>
+          <t>Create article with empty title</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>1. Upload cover
-2. Body diisi
-3. Judul kosong
-4. Klik Publish</t>
+2. Fill body
+3. Leave title empty
+4. Click Publish</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Validasi: judul wajib diisi</t>
+          <t>Validation: title is required</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1076,30 +1077,30 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Membuat artikel tanpa body</t>
+          <t>Create article without body</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>1. Isi judul
+          <t>1. Fill title
 2. Upload cover
-3. Body kosong
+3. Leave body empty
 4. Submit</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Validasi: body tidak boleh kosong</t>
+          <t>Validation: body cannot be empty</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1126,27 +1127,27 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Melihat detail artikel</t>
+          <t>View article detail</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Ada artikel published</t>
+          <t>Published article exists</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>1. Klik card artikel di feed</t>
+          <t>1. Click article card in feed</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Halaman detail: title, body, cover, author, komen</t>
+          <t>Detail page: title, body, cover, author, comments</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1173,27 +1174,27 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Like artikel</t>
+          <t>Like an article</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Login, ada artikel</t>
+          <t>Logged in, article exists</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol like</t>
+          <t>Click like button</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Icon berubah, count +1</t>
+          <t>Icon changes, count +1</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -1220,27 +1221,27 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Unlike artikel</t>
+          <t>Unlike an article</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Login, sudah like</t>
+          <t>Logged in, already liked</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol like lagi</t>
+          <t>Click like button again</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Icon kembali, count -1</t>
+          <t>Icon reverts, count -1</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1267,27 +1268,27 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Save artikel</t>
+          <t>Save an article</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol save</t>
+          <t>Click save button</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Artikel tersimpan</t>
+          <t>Article saved</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1314,29 +1315,29 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Tambah komentar</t>
+          <t>Add comment</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in, article exists</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>1. Scroll ke komentar
-2. Tulis komentar
+          <t>1. Scroll to comments
+2. Write comment
 3. Submit</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Komentar muncul di thread</t>
+          <t>Comment appears in thread</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1363,27 +1364,27 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Komentar dengan konten kosong</t>
+          <t>Add empty comment</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1. Klik submit tanpa isi komentar</t>
+          <t>1. Click submit without typing</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Validasi: komentar tidak boleh kosong</t>
+          <t>Validation: comment cannot be empty</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1410,27 +1411,27 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Hapus komentar sendiri</t>
+          <t>Delete own comment</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Login, punya komentar</t>
+          <t>Logged in, owns a comment</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Klik hapus pada komentar sendiri</t>
+          <t>Click delete on own comment</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Komentar terhapus</t>
+          <t>Comment deleted</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1457,27 +1458,27 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Tab My Articles</t>
+          <t>My Articles tab</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Login, punya artikel</t>
+          <t>Logged in, has own articles</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>1. Buka tab 'My Articles'</t>
+          <t>1. Open 'My Articles' tab</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Hanya artikel milik sendiri tampil</t>
+          <t>Only user's own articles displayed</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1504,27 +1505,27 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Melihat daftar lobby</t>
+          <t>View lobby list</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>1. Buka Team Builder tab</t>
+          <t>1. Open Team Builder tab</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Lobby cards tampil (nama, kompetisi, role, deadline)</t>
+          <t>Lobby cards displayed (name, competition, roles, deadline)</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1551,27 +1552,27 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Filter lobby by kompetisi</t>
+          <t>Filter lobbies by competition</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Ada data lobby</t>
+          <t>Lobby data exists</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Pilih filter kompetisi</t>
+          <t>Select competition filter</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Lobby terfilter</t>
+          <t>Lobbies filtered</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1598,27 +1599,27 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Filter lobby by universitas</t>
+          <t>Filter lobbies by university</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Ada data lobby</t>
+          <t>Lobby data exists</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Pilih filter universitas</t>
+          <t>Select university filter</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Lobby dari universitas tertentu</t>
+          <t>Lobbies from selected university</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1645,31 +1646,31 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Buat lobby (catalog mode)</t>
+          <t>Create lobby (catalog mode)</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>1. Klik 'Buat Lobby'
-2. Step 1: Pilih kompetisi dari katalog
-3. Step 2: Isi nama tim, deskripsi
-4. Step 3: Atur roles &amp; deadline
+          <t>1. Click 'Create Lobby'
+2. Step 1: Pick competition from catalog
+3. Step 2: Fill team name, description
+4. Step 3: Set roles &amp; deadline
 5. Submit</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Lobby berhasil dibuat</t>
+          <t>Lobby created successfully</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1696,29 +1697,29 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Buat lobby (manual mode)</t>
+          <t>Create lobby (manual mode)</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>1. Pilih manual mode
-2. Input nama kompetisi manual
-3-5. Sama seperti catalog</t>
+          <t>1. Select manual mode
+2. Input competition name manually
+3-5. Same as catalog flow</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Lobby manual berhasil</t>
+          <t>Manual lobby created</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -1745,29 +1746,29 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Validasi - nama tim kosong</t>
+          <t>Validation — empty team name</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>1. Buka create lobby
-2. Kosongi nama tim
+          <t>1. Open create lobby
+2. Leave team name empty
 3. Submit</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Validasi: nama tim wajib</t>
+          <t>Validation: team name required</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1794,28 +1795,28 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Validasi - deadline lewat</t>
+          <t>Validation — past deadline</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>1. Set deadline di masa lalu
+          <t>1. Set deadline in the past
 2. Submit</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Validasi: deadline harus di masa depan</t>
+          <t>Validation: deadline must be in the future</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1842,28 +1843,28 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Validasi - role kosong</t>
+          <t>Validation — no roles selected</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>1. Tidak pilih role yang dicari
+          <t>1. Don't select any roles
 2. Submit</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Validasi: minimal 1 role</t>
+          <t>Validation: at least 1 role required</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1890,27 +1891,27 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Melihat detail lobby</t>
+          <t>View lobby detail</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Ada lobby</t>
+          <t>Lobby exists</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Klik lobby card</t>
+          <t>Click lobby card</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Detail: anggota, roles, deadline, status, tombol apply</t>
+          <t>Detail: members, roles, deadline, status, apply button</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -1937,27 +1938,27 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Apply ke lobby</t>
+          <t>Apply to lobby</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Login, bukan owner</t>
+          <t>Logged in, not the owner</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Klik Apply</t>
+          <t>Click Apply button</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Application terkirim, status pending</t>
+          <t>Application sent, status pending</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -1984,27 +1985,27 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Apply ke lobby penuh</t>
+          <t>Apply to full lobby</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Lobby sudah penuh</t>
+          <t>Lobby is full</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Klik Apply</t>
+          <t>Click Apply</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Error: lobby full / notifikasi</t>
+          <t>Error: lobby is full / notification</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -2031,22 +2032,22 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Apply ke lobby sendiri (owner)</t>
+          <t>Apply to own lobby (owner)</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Login sebagai owner</t>
+          <t>Logged in as owner</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Klik Apply di lobby sendiri</t>
+          <t>Click Apply on own lobby</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Tombol apply tidak muncul atau disable</t>
+          <t>Apply button hidden or disabled</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -2078,28 +2079,28 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Review applicant - approve</t>
+          <t>Review applicant — approve</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Login sebagai owner, ada applicant</t>
+          <t>Logged in as owner, applicant exists</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>1. Buka lobby
+          <t>1. Open lobby
 2. Approve applicant</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Applicant masuk anggota</t>
+          <t>Applicant added as member</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -2126,12 +2127,12 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Review applicant - reject</t>
+          <t>Review applicant — reject</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Login sebagai owner</t>
+          <t>Logged in as owner</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -2141,12 +2142,12 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Applicant ditolak</t>
+          <t>Applicant rejected</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2173,27 +2174,27 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Review applicant bukan owner</t>
+          <t>Review applicant (not owner)</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Login bukan owner</t>
+          <t>Logged in, not the owner</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Coba review applicant</t>
+          <t>Try to review applicant</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Tombol review tidak muncul</t>
+          <t>Review button not visible</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2220,27 +2221,27 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Hapus lobby (owner)</t>
+          <t>Delete lobby (owner)</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Login sebagai owner</t>
+          <t>Logged in as owner</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Klik hapus lobby</t>
+          <t>Click delete lobby</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Lobby terhapus</t>
+          <t>Lobby deleted</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2267,27 +2268,27 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Hapus lobby (bukan owner)</t>
+          <t>Delete lobby (not owner)</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Login bukan owner</t>
+          <t>Logged in, not the owner</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Coba hapus lobby milik orang lain</t>
+          <t>Try to delete another's lobby</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Tombol hapus tidak muncul / error</t>
+          <t>Delete button hidden / error</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2319,22 +2320,22 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Login sebagai anggota</t>
+          <t>Logged in as member</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Klik request leave</t>
+          <t>Click request leave</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Request terkirim ke owner</t>
+          <t>Leave request sent to owner</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -2361,28 +2362,28 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Buka form add class/bootcamp</t>
+          <t>Open add class/bootcamp form</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Login admin</t>
+          <t>Logged in as admin</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>1. Buka admin dashboard
-2. Klik Add Bootcamp/Class</t>
+          <t>1. Open admin dashboard
+2. Click Add Bootcamp/Class</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Form tampil, ada opsi selection</t>
+          <t>Form displayed with selection toggle option</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2409,12 +2410,12 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Aktifkan selection toggle</t>
+          <t>Enable selection toggle</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Login admin, form add</t>
+          <t>Admin logged in, form open</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2424,12 +2425,12 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Question builder muncul</t>
+          <t>Question builder appears</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2456,27 +2457,27 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Tambah pertanyaan selection</t>
+          <t>Add selection question</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Selection aktif</t>
+          <t>Selection enabled</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Klik 'Tambah Pertanyaan'</t>
+          <t>Click 'Add Question'</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Input field pertanyaan baru</t>
+          <t>New question input field added</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2503,30 +2504,30 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Isi semua field selection</t>
+          <t>Fill all selection fields</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Selection aktif</t>
+          <t>Selection enabled</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>1. Isi judul form
-2. Isi deskripsi
-3. Tambah 3 pertanyaan
-4. Simpan</t>
+          <t>1. Fill form title
+2. Fill description
+3. Add 3 questions
+4. Save</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Semua tersimpan</t>
+          <t>All data saved successfully</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -2553,27 +2554,27 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Validasi - judul form kosong</t>
+          <t>Validation — empty form title</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Selection aktif</t>
+          <t>Selection enabled</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Kosongi judul, isi pertanyaan, submit</t>
+          <t>Leave title empty, add questions, submit</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Error: judul wajib diisi</t>
+          <t>Error: title is required</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2600,27 +2601,27 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Validasi - tanpa pertanyaan</t>
+          <t>Validation — no questions added</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Selection aktif</t>
+          <t>Selection enabled</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Isi judul, 0 pertanyaan, submit</t>
+          <t>Fill title, 0 questions, submit</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Error: minimal 1 pertanyaan</t>
+          <t>Error: at least 1 question required</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2647,27 +2648,27 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Hapus pertanyaan</t>
+          <t>Delete a question</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Ada 2+ pertanyaan</t>
+          <t>2+ questions exist</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Klik hapus pada satu pertanyaan</t>
+          <t>Click delete on one question</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>Pertanyaan terhapus</t>
+          <t>Question removed from list</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -2694,27 +2695,27 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Reorder pertanyaan (drag)</t>
+          <t>Reorder questions (drag)</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Ada 2+ pertanyaan</t>
+          <t>2+ questions exist</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Drag &amp; drop urutan</t>
+          <t>Drag &amp; drop to reorder</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>Urutan berubah</t>
+          <t>Order changed</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2741,12 +2742,12 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Nonaktifkan selection</t>
+          <t>Disable selection</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Selection aktif</t>
+          <t>Selection is enabled</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2756,12 +2757,12 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Question builder hilang</t>
+          <t>Question builder disappears</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2788,28 +2789,28 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Edit selection form</t>
+          <t>Edit existing selection form</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Ada data class dengan selection</t>
+          <t>Bootcamp with selection exists</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
           <t>1. Edit bootcamp
-2. Lihat selection form</t>
+2. Check selection form</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Data selection sebelumnya muncul</t>
+          <t>Previous selection data pre-filled</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -2836,23 +2837,23 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>User daftar dengan selection</t>
+          <t>User sees selection form on registration</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Ada bootcamp dengan selection</t>
+          <t>Bootcamp with selection exists</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>1. User klik daftar bootcamp
-2. Lihat form</t>
+          <t>1. User clicks register for bootcamp
+2. View form</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Form seleksi muncul sebelum konfirmasi</t>
+          <t>Selection form shown before confirmation</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
@@ -2884,28 +2885,28 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>User submit form selection</t>
+          <t>User submits selection form</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Ada bootcamp+selection</t>
+          <t>Bootcamp with selection exists</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>1. Isi form seleksi
+          <t>1. Fill selection form
 2. Submit</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Pendaftaran berhasil</t>
+          <t>Registration successful</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2933,8 +2934,8 @@
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
@@ -2943,12 +2944,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>TC ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Modul</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -2963,7 +2964,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Skenario</t>
+          <t>Scenario</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -2983,7 +2984,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Tipe</t>
+          <t>Type</t>
         </is>
       </c>
     </row>
@@ -3023,12 +3024,12 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Data artikel array</t>
+          <t>Articles array</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3068,12 +3069,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Artikel sesuai search</t>
+          <t>Matching articles</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3113,12 +3114,12 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Artikel terfilter</t>
+          <t>Filtered articles</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3146,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Trending articles</t>
+          <t>Get trending articles</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -3158,12 +3159,12 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Array trending articles</t>
+          <t>Trending array</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3203,12 +3204,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Array tags (id, name)</t>
+          <t>Tags array (id, name)</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3248,12 +3249,12 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Data artikel + author</t>
+          <t>Article data + author</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3286,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>slug-tidak-ada</t>
+          <t>non-existent-slug</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
@@ -3298,7 +3299,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -3338,12 +3339,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Array comments</t>
+          <t>Comments array</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3371,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Login valid</t>
+          <t>Login with valid credentials</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -3388,7 +3389,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3415,7 +3416,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Login wrong password</t>
+          <t>Login with wrong password</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -3433,7 +3434,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3461,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Login non-existent email</t>
+          <t>Login with non-existent email</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -3478,7 +3479,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -3505,7 +3506,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Login empty fields</t>
+          <t>Login with empty fields</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -3523,7 +3524,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3569,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -3608,12 +3609,12 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>User articles array</t>
+          <t>User's articles array</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3641,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Saved articles</t>
+          <t>Get saved articles</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -3658,7 +3659,7 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3686,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Following articles</t>
+          <t>Get following feed</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -3703,7 +3704,7 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3749,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3794,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3839,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -3883,7 +3884,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3929,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3974,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4019,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4063,7 +4064,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -4090,7 +4091,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Like article</t>
+          <t>Like an article</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -4108,7 +4109,7 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4136,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Unlike article</t>
+          <t>Unlike an article</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -4153,7 +4154,7 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4181,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Save article</t>
+          <t>Save an article</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -4198,7 +4199,7 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4225,7 +4226,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Unsave article</t>
+          <t>Unsave an article</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -4243,7 +4244,7 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4275,7 +4276,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>{"content":"Bagus!"}</t>
+          <t>{"content":"Great article!"}</t>
         </is>
       </c>
       <c r="G30" s="3" t="n">
@@ -4288,7 +4289,7 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4316,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Add comment (empty)</t>
+          <t>Add empty comment</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -4333,7 +4334,7 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4379,7 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4406,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Delete others comment</t>
+          <t>Delete others' comment</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -4423,7 +4424,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4469,7 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4514,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4558,7 +4559,7 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4604,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Get all lobbies (auth)</t>
+          <t>Get all lobbies with filters</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -4648,7 +4649,7 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4693,7 +4694,7 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4733,12 +4734,12 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>Lobby detail</t>
+          <t>Lobby detail object</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4784,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4816,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>{"name":"Tim Olimpiade","competition_id":1,"team_size":3,"roles":["Programmer"],"deadline":"2026-08-01"}</t>
+          <t>{"name":"Olimpiade Team","competition_id":1,"team_size":3,"roles":["Programmer"],"deadline":"2026-08-01"}</t>
         </is>
       </c>
       <c r="G42" s="3" t="n">
@@ -4828,7 +4829,7 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4874,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4919,7 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4964,7 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4991,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Delete others lobby</t>
+          <t>Delete others' lobby</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -5008,7 +5009,7 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5041,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>{"cover_letter":"Saya tertarik"}</t>
+          <t>{"cover_letter":"I want to join!"}</t>
         </is>
       </c>
       <c r="G47" s="3" t="n">
@@ -5053,7 +5054,7 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5081,7 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Apply twice</t>
+          <t>Apply twice (double)</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -5098,7 +5099,7 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -5143,7 +5144,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5189,7 @@
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5233,7 +5234,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5279,7 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5323,7 +5324,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5368,7 +5369,7 @@
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5414,7 @@
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5440,7 +5441,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>My active room</t>
+          <t>Get my active room</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -5458,7 +5459,7 @@
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5504,7 @@
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5535,7 +5536,7 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>{"name":"Lomba Baru","selection_enabled":true,"selection_form_title":"Seleksi","selection_questions":[{"question":"Alasan ikut?"}]}</t>
+          <t>{"name":"New Competition","selection_enabled":true,"selection_form_title":"Selection","selection_questions":[{"question":"Why join?"}]}</t>
         </is>
       </c>
       <c r="G58" s="3" t="n">
@@ -5548,7 +5549,7 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5581,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>{"name":"Lomba Baru 2","selection_enabled":false}</t>
+          <t>{"name":"Competition 2","selection_enabled":false}</t>
         </is>
       </c>
       <c r="G59" s="3" t="n">
@@ -5593,7 +5594,7 @@
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5639,7 @@
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5666,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Add with empty questions when enabled</t>
+          <t>Enable selection with empty questions</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -5683,7 +5684,7 @@
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Negative</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5716,7 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>{"selection_enabled":true,"selection_form_title":"Updated Seleksi"}</t>
+          <t>{"selection_enabled":true,"selection_form_title":"Updated Selection"}</t>
         </is>
       </c>
       <c r="G62" s="3" t="n">
@@ -5728,7 +5729,7 @@
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Positive</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: English headers + Status column in XLSX
- Changed all column headers to English
- Added Status column (Pass/Fail/Pending/Not Tested) to both Manual + API sheets
- Ready for execution tracking
</commit_message>
<xml_diff>
--- a/projects/akademi-competition/test-cases.xlsx
+++ b/projects/akademi-competition/test-cases.xlsx
@@ -13,8 +13,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manual Test Cases'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API Test Cases'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manual Test Cases'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API Test Cases'!$A$1:$J$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -479,7 +479,6 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -656,24 +655,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="35" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TC ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -714,6 +714,11 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -740,18 +745,18 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Logged in, articles exist in DB</t>
+          <t>Logged in, has published articles</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>1. Open /user/social-forum
-2. For You tab is active</t>
+2. For You tab active</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Article cards displayed with infinite scroll</t>
+          <t>Articles displayed as cards, infinite scroll works</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -764,6 +769,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -799,7 +805,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Matching articles displayed</t>
+          <t>Articles matching keyword displayed</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -812,6 +818,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -836,12 +843,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Tags and tagged articles exist</t>
+          <t>Tags &amp; articles with tags exist</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>1. Click filter button
+          <t>1. Click filter tag
 2. Select 1+ tags</t>
         </is>
       </c>
@@ -860,6 +867,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -907,6 +915,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -926,7 +935,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Create a new article</t>
+          <t>Create new article</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -936,7 +945,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>1. Click 'Create Article'
+          <t>1. Click 'Buat Artikel'
 2. Fill title
 3. Fill body (rich text)
 4. Upload cover image
@@ -960,6 +969,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -995,7 +1005,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Validation: cover image is required</t>
+          <t>Validation: cover image required</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1008,6 +1018,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1058,6 +1069,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1108,6 +1120,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1155,6 +1168,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1174,7 +1188,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Like an article</t>
+          <t>Like article</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1202,6 +1216,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1221,7 +1236,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Unlike an article</t>
+          <t>Unlike article</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1249,6 +1264,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1268,7 +1284,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Save an article</t>
+          <t>Save article</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1296,6 +1312,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1320,7 +1337,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Logged in, article exists</t>
+          <t>Logged in</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1345,6 +1362,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1374,7 +1392,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>1. Click submit without typing</t>
+          <t>1. Click submit without filling comment</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1392,6 +1410,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1416,7 +1435,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Logged in, owns a comment</t>
+          <t>Logged in, has comment</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1439,6 +1458,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1463,7 +1483,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Logged in, has own articles</t>
+          <t>Logged in, has articles</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1486,6 +1506,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1520,7 +1541,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Lobby cards displayed (name, competition, roles, deadline)</t>
+          <t>Lobby cards displayed (name, competition, role, deadline)</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1533,6 +1554,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1552,7 +1574,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Filter lobbies by competition</t>
+          <t>Filter lobby by competition</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1567,7 +1589,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Lobbies filtered</t>
+          <t>Lobby filtered by competition</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1580,6 +1602,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1599,7 +1622,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Filter lobbies by university</t>
+          <t>Filter lobby by university</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1614,7 +1637,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Lobbies from selected university</t>
+          <t>Lobby filtered by university</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1627,6 +1650,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1656,8 +1680,8 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>1. Click 'Create Lobby'
-2. Step 1: Pick competition from catalog
+          <t>1. Click 'Buat Lobby'
+2. Step 1: Select competition from catalog
 3. Step 2: Fill team name, description
 4. Step 3: Set roles &amp; deadline
 5. Submit</t>
@@ -1678,6 +1702,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1709,12 +1734,12 @@
         <is>
           <t>1. Select manual mode
 2. Input competition name manually
-3-5. Same as catalog flow</t>
+3-5. Same as catalog</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Manual lobby created</t>
+          <t>Manual lobby created successfully</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -1727,6 +1752,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1746,7 +1772,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Validation — empty team name</t>
+          <t>Validation - empty team name</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -1776,6 +1802,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1795,7 +1822,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Validation — past deadline</t>
+          <t>Validation - past deadline</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1824,6 +1851,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1843,7 +1871,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Validation — no roles selected</t>
+          <t>Validation - no role selected</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1853,7 +1881,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>1. Don't select any roles
+          <t>1. Don't select any role
 2. Submit</t>
         </is>
       </c>
@@ -1872,6 +1900,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1919,6 +1948,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1943,12 +1973,12 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Logged in, not the owner</t>
+          <t>Logged in, not owner</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Click Apply button</t>
+          <t>Click Apply</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1966,6 +1996,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2000,7 +2031,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Error: lobby is full / notification</t>
+          <t>Error: lobby full / notification</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -2013,6 +2044,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2060,6 +2092,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -2079,7 +2112,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Review applicant — approve</t>
+          <t>Review applicant - approve</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -2108,6 +2141,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -2127,7 +2161,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Review applicant — reject</t>
+          <t>Review applicant - reject</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -2155,6 +2189,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2179,7 +2214,7 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Logged in, not the owner</t>
+          <t>Logged in as non-owner</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -2202,6 +2237,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -2249,6 +2285,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2273,7 +2310,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Logged in, not the owner</t>
+          <t>Logged in as non-owner</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -2283,7 +2320,7 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Delete button hidden / error</t>
+          <t>Delete button not visible / error</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2296,6 +2333,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2330,7 +2368,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Leave request sent to owner</t>
+          <t>Request sent to owner</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -2343,6 +2381,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -2378,7 +2417,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Form displayed with selection toggle option</t>
+          <t>Form displayed with selection option</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -2391,6 +2430,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2415,7 +2455,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Admin logged in, form open</t>
+          <t>Logged in as admin, form open</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2438,6 +2478,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2467,7 +2508,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Click 'Add Question'</t>
+          <t>Click 'Tambah Pertanyaan'</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -2485,6 +2526,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2522,7 +2564,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>All data saved successfully</t>
+          <t>All fields saved successfully</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2535,6 +2577,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2554,7 +2597,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Validation — empty form title</t>
+          <t>Validation - empty form title</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
@@ -2564,7 +2607,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Leave title empty, add questions, submit</t>
+          <t>Leave title empty, fill questions, submit</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -2582,6 +2625,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2601,7 +2645,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Validation — no questions added</t>
+          <t>Validation - no questions</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2629,6 +2673,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2648,7 +2693,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Delete a question</t>
+          <t>Delete question</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2676,6 +2721,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2723,6 +2769,7 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="J43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -2747,7 +2794,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Selection is enabled</t>
+          <t>Selection enabled</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2757,7 +2804,7 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Question builder disappears</t>
+          <t>Question builder hidden</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -2770,6 +2817,7 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="J44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2789,23 +2837,23 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Edit existing selection form</t>
+          <t>Edit selection form</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Bootcamp with selection exists</t>
+          <t>Class with selection exists</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
           <t>1. Edit bootcamp
-2. Check selection form</t>
+2. View selection form</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Previous selection data pre-filled</t>
+          <t>Previous selection data displayed</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -2818,6 +2866,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -2837,7 +2886,7 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>User sees selection form on registration</t>
+          <t>User registers with selection</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2847,7 +2896,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>1. User clicks register for bootcamp
+          <t>1. User clicks register
 2. View form</t>
         </is>
       </c>
@@ -2866,6 +2915,7 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2890,7 +2940,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Bootcamp with selection exists</t>
+          <t>Bootcamp+selection exists</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -2914,9 +2964,10 @@
           <t>High</t>
         </is>
       </c>
+      <c r="J47" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2927,24 +2978,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TC ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -2985,6 +3037,11 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3081,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Articles array</t>
+          <t>Articles data array</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -3032,6 +3089,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -3077,6 +3135,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -3122,6 +3181,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3159,7 +3219,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Trending array</t>
+          <t>Trending articles array</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -3167,6 +3227,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -3212,6 +3273,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3249,7 +3311,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Article data + author</t>
+          <t>Article + author data</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -3257,6 +3319,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -3286,7 +3349,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>non-existent-slug</t>
+          <t>slug-tidak-ada</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
@@ -3302,6 +3365,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3347,6 +3411,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -3371,7 +3436,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Login with valid credentials</t>
+          <t>Login valid</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -3392,6 +3457,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -3416,7 +3482,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Login with wrong password</t>
+          <t>Login wrong password</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -3437,6 +3503,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -3461,7 +3528,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Login with non-existent email</t>
+          <t>Login non-existent email</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -3482,6 +3549,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -3506,7 +3574,7 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Login with empty fields</t>
+          <t>Login empty fields</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -3527,6 +3595,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -3572,6 +3641,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3609,7 +3679,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>User's articles array</t>
+          <t>User articles array</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -3617,6 +3687,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -3662,6 +3733,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3686,7 +3758,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Get following feed</t>
+          <t>Get following articles</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -3707,6 +3779,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -3752,6 +3825,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -3797,6 +3871,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -3842,6 +3917,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -3887,6 +3963,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -3932,6 +4009,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -3977,6 +4055,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -4022,6 +4101,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -4067,6 +4147,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -4091,7 +4172,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Like an article</t>
+          <t>Like article</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -4112,6 +4193,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -4136,7 +4218,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Unlike an article</t>
+          <t>Unlike article</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -4157,6 +4239,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -4181,7 +4264,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Save an article</t>
+          <t>Save article</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -4202,6 +4285,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -4226,7 +4310,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Unsave an article</t>
+          <t>Unsave article</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -4247,6 +4331,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -4292,6 +4377,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -4316,7 +4402,7 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Add empty comment</t>
+          <t>Add comment (empty)</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -4337,6 +4423,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -4382,6 +4469,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -4406,7 +4494,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Delete others' comment</t>
+          <t>Delete others comment</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -4427,6 +4515,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -4472,6 +4561,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -4517,6 +4607,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -4562,6 +4653,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -4607,6 +4699,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -4631,7 +4724,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Get all lobbies with filters</t>
+          <t>Get all lobbies (auth)</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -4652,6 +4745,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -4697,6 +4791,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -4734,7 +4829,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>Lobby detail object</t>
+          <t>Lobby detail</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -4742,6 +4837,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -4787,6 +4883,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -4816,7 +4913,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>{"name":"Olimpiade Team","competition_id":1,"team_size":3,"roles":["Programmer"],"deadline":"2026-08-01"}</t>
+          <t>{"name":"Team Olimpiade","competition_id":1,"team_size":3,"roles":["Programmer"],"deadline":"2026-08-01"}</t>
         </is>
       </c>
       <c r="G42" s="3" t="n">
@@ -4832,6 +4929,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -4877,6 +4975,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -4922,6 +5021,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -4967,6 +5067,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -4991,7 +5092,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Delete others' lobby</t>
+          <t>Delete others lobby</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -5012,6 +5113,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -5041,7 +5143,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>{"cover_letter":"I want to join!"}</t>
+          <t>{"cover_letter":"I am interested"}</t>
         </is>
       </c>
       <c r="G47" s="3" t="n">
@@ -5057,6 +5159,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -5081,7 +5184,7 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Apply twice (double)</t>
+          <t>Apply twice</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -5102,6 +5205,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -5147,6 +5251,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -5192,6 +5297,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -5237,6 +5343,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -5282,6 +5389,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -5327,6 +5435,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -5372,6 +5481,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J54" s="4" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -5417,6 +5527,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -5441,7 +5552,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Get my active room</t>
+          <t>My active room</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -5462,6 +5573,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -5507,6 +5619,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -5552,6 +5665,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -5581,7 +5695,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>{"name":"Competition 2","selection_enabled":false}</t>
+          <t>{"name":"New Comp 2","selection_enabled":false}</t>
         </is>
       </c>
       <c r="G59" s="3" t="n">
@@ -5597,6 +5711,7 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -5642,6 +5757,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -5666,12 +5782,12 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Enable selection with empty questions</t>
+          <t>Add with empty questions when enabled</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>{"name":"Lomba","selection_enabled":true,"questions":[]}</t>
+          <t>{"name":"Comp","selection_enabled":true,"questions":[]}</t>
         </is>
       </c>
       <c r="G61" s="4" t="n">
@@ -5679,7 +5795,7 @@
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>Validation failed</t>
+          <t>Validation error</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
@@ -5687,6 +5803,7 @@
           <t>Negative</t>
         </is>
       </c>
+      <c r="J61" s="4" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -5732,9 +5849,10 @@
           <t>Positive</t>
         </is>
       </c>
+      <c r="J62" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: English headers + Result column for all XLSX
- Semua test cases: headers pake English
- Column Result (ungu) buat diisi pass/fail pas testing
- Arteri: Test Cases → Type, Precondition, Notes, Result
- IFL: same format
- Akademi: Manual + API with Result column
- Color coding (green=positive, red=negative, yellow=edge) tetap
- Auto filter + frozen header di semua sheet
</commit_message>
<xml_diff>
--- a/projects/akademi-competition/test-cases.xlsx
+++ b/projects/akademi-competition/test-cases.xlsx
@@ -13,8 +13,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manual Test Cases'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API Test Cases'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Manual Test Cases'!$A$1:$J$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'API Test Cases'!$A$1:$J$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38,7 +38,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +69,30 @@
         <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9333EA"/>
+        <bgColor rgb="FF9333EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009333EA"/>
+        <bgColor rgb="009333EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
+        <bgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -88,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -104,6 +128,36 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -659,15 +713,15 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -716,9 +770,9 @@
           <t>Priority</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>Result</t>
         </is>
       </c>
     </row>
@@ -769,7 +823,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="J2" s="11" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -818,7 +872,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="11" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -867,7 +921,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="J4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -915,7 +969,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
+      <c r="J5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -969,84 +1023,84 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
+      <c r="J6" s="11" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>A-C-06</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Create</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Create article without cover image</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Logged in</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>1. Fill all fields except cover
 2. Click Publish</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>Validation: cover image required</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="J7" s="13" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>A-C-07</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Create</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Create article with empty title</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Logged in</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>1. Upload cover
 2. Fill body
@@ -1054,50 +1108,50 @@
 4. Click Publish</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>Validation: title is required</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="J8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>A-C-08</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Create</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Create article without body</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Logged in</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>1. Fill title
 2. Upload cover
@@ -1105,22 +1159,22 @@
 4. Submit</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>Validation: body cannot be empty</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr"/>
+      <c r="J9" s="13" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1168,7 +1222,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1216,7 +1270,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1264,7 +1318,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1312,7 +1366,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr"/>
+      <c r="J13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1362,55 +1416,55 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr"/>
+      <c r="J14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>A-C-14</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Add empty comment</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Logged in</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>1. Click submit without filling comment</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>Validation: comment cannot be empty</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I15" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr"/>
+      <c r="J15" s="13" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1458,7 +1512,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="J16" s="11" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1506,7 +1560,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr"/>
+      <c r="J17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1554,7 +1608,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr"/>
+      <c r="J18" s="11" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1602,7 +1656,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr"/>
+      <c r="J19" s="11" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1650,7 +1704,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr"/>
+      <c r="J20" s="11" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1702,7 +1756,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr"/>
+      <c r="J21" s="11" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1752,155 +1806,155 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="J22" s="11" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>T-C-06</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>Create Lobby</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Validation - empty team name</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Logged in</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>1. Open create lobby
 2. Leave team name empty
 3. Submit</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Validation: team name required</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I23" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr"/>
+      <c r="J23" s="13" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>T-C-07</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="12" t="inlineStr">
         <is>
           <t>Create Lobby</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Validation - past deadline</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>Logged in</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="12" t="inlineStr">
         <is>
           <t>1. Set deadline in the past
 2. Submit</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>Validation: deadline must be in the future</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H24" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I24" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr"/>
+      <c r="J24" s="13" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>T-C-08</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Create Lobby</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Validation - no role selected</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Logged in</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>1. Don't select any role
 2. Submit</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>Validation: at least 1 role required</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H25" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I25" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr"/>
+      <c r="J25" s="13" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1948,7 +2002,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr"/>
+      <c r="J26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1996,103 +2050,103 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr"/>
+      <c r="J27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>T-C-11</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>Join</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Apply to full lobby</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="12" t="inlineStr">
         <is>
           <t>Lobby is full</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Click Apply</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>Error: lobby full / notification</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H28" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I28" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr"/>
+      <c r="J28" s="13" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>T-C-12</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>Join</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Apply to own lobby (owner)</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>Logged in as owner</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>Click Apply on own lobby</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Apply button hidden or disabled</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H29" s="14" t="inlineStr">
         <is>
           <t>Edge</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I29" s="14" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr"/>
+      <c r="J29" s="15" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -2141,7 +2195,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr"/>
+      <c r="J30" s="11" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -2189,55 +2243,55 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr"/>
+      <c r="J31" s="11" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>T-C-15</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="12" t="inlineStr">
         <is>
           <t>Manage</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>Review applicant (not owner)</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="12" t="inlineStr">
         <is>
           <t>Logged in as non-owner</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="12" t="inlineStr">
         <is>
           <t>Try to review applicant</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="12" t="inlineStr">
         <is>
           <t>Review button not visible</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H32" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I32" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr"/>
+      <c r="J32" s="13" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -2285,55 +2339,55 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr"/>
+      <c r="J33" s="11" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>T-C-17</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Manage</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Delete lobby (not owner)</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="12" t="inlineStr">
         <is>
           <t>Logged in as non-owner</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="12" t="inlineStr">
         <is>
           <t>Try to delete another's lobby</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G34" s="12" t="inlineStr">
         <is>
           <t>Delete button not visible / error</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H34" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I34" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr"/>
+      <c r="J34" s="13" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2381,7 +2435,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr"/>
+      <c r="J35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -2430,7 +2484,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J36" s="3" t="inlineStr"/>
+      <c r="J36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2478,7 +2532,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J37" s="3" t="inlineStr"/>
+      <c r="J37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2526,7 +2580,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J38" s="3" t="inlineStr"/>
+      <c r="J38" s="11" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2577,103 +2631,103 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J39" s="3" t="inlineStr"/>
+      <c r="J39" s="11" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t>S-C-05</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>Selection Form</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>Admin Config</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>Validation - empty form title</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E40" s="12" t="inlineStr">
         <is>
           <t>Selection enabled</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F40" s="12" t="inlineStr">
         <is>
           <t>Leave title empty, fill questions, submit</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="G40" s="12" t="inlineStr">
         <is>
           <t>Error: title is required</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="H40" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="I40" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr"/>
+      <c r="J40" s="13" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>S-C-06</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>Selection Form</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>Admin Config</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>Validation - no questions</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Selection enabled</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F41" s="12" t="inlineStr">
         <is>
           <t>Fill title, 0 questions, submit</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="G41" s="12" t="inlineStr">
         <is>
           <t>Error: at least 1 question required</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="H41" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I41" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr"/>
+      <c r="J41" s="13" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2721,7 +2775,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J42" s="3" t="inlineStr"/>
+      <c r="J42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2769,7 +2823,7 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="J43" s="3" t="inlineStr"/>
+      <c r="J43" s="11" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -2817,7 +2871,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="J44" s="3" t="inlineStr"/>
+      <c r="J44" s="11" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2866,56 +2920,56 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J45" s="3" t="inlineStr"/>
+      <c r="J45" s="11" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>S-C-11</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>Selection Form</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>User View</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>User registers with selection</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E46" s="14" t="inlineStr">
         <is>
           <t>Bootcamp with selection exists</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F46" s="14" t="inlineStr">
         <is>
           <t>1. User clicks register
 2. View form</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="G46" s="14" t="inlineStr">
         <is>
           <t>Selection form shown before confirmation</t>
         </is>
       </c>
-      <c r="H46" s="5" t="inlineStr">
+      <c r="H46" s="14" t="inlineStr">
         <is>
           <t>Edge</t>
         </is>
       </c>
-      <c r="I46" s="5" t="inlineStr">
+      <c r="I46" s="14" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J46" s="5" t="inlineStr"/>
+      <c r="J46" s="15" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2964,10 +3018,10 @@
           <t>High</t>
         </is>
       </c>
-      <c r="J47" s="3" t="inlineStr"/>
+      <c r="J47" s="11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:J47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2981,16 +3035,16 @@
   <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3039,9 +3093,9 @@
           <t>Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>Result</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3143,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="J2" s="11" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -3135,7 +3189,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
+      <c r="J3" s="11" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -3181,7 +3235,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="J4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3227,7 +3281,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
+      <c r="J5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -3273,7 +3327,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
+      <c r="J6" s="11" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3319,53 +3373,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>API-PUB-07</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Public</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>/articles/:slug</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Article detail (invalid slug)</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>slug-tidak-ada</t>
         </is>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="12" t="n">
         <v>404</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>Not found</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="J8" s="13" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3411,7 +3465,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="J9" s="11" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -3457,191 +3511,191 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>API-AUTH-02</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Auth</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>/auth/login</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Login wrong password</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>{"email":"user@test.com","password":"wrong"}</t>
         </is>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="12" t="n">
         <v>401</v>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>Unauthorized</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr"/>
+      <c r="J11" s="13" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>API-AUTH-03</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Auth</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>/auth/login</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>Login non-existent email</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>{"email":"noone@test.com","password":"test"}</t>
         </is>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="12" t="n">
         <v>401</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>Unauthorized</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="J12" s="13" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>API-AUTH-04</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Auth</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>/auth/login</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Login empty fields</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
         <is>
           <t>Validation error</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I13" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr"/>
+      <c r="J13" s="13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>API-ART-01</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>/users/articles</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>My articles (no auth)</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="12" t="n">
         <v>401</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>Unauthorized</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I14" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr"/>
+      <c r="J14" s="13" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3687,7 +3741,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr"/>
+      <c r="J15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -3733,7 +3787,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="J16" s="11" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3779,7 +3833,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr"/>
+      <c r="J17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -3825,145 +3879,145 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr"/>
+      <c r="J18" s="11" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>API-ART-06</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>/users/articles</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Create article (no cover)</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>multipart without cover_image</t>
         </is>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="G19" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="12" t="inlineStr">
         <is>
           <t>Cover image required</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I19" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr"/>
+      <c r="J19" s="13" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>API-ART-07</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="12" t="inlineStr">
         <is>
           <t>/users/articles</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Create article (no title)</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="12" t="inlineStr">
         <is>
           <t>multipart without title</t>
         </is>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="G20" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="12" t="inlineStr">
         <is>
           <t>Title required</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I20" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="J20" s="13" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>API-ART-08</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>/users/articles</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Create article (no auth)</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>multipart valid but no token</t>
         </is>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="G21" s="12" t="n">
         <v>401</v>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="12" t="inlineStr">
         <is>
           <t>Unauthorized</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I21" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr"/>
+      <c r="J21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -4009,53 +4063,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="J22" s="11" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>API-ART-10</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>/users/articles/:id</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Update article (not owner)</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>multipart: updated title</t>
         </is>
       </c>
-      <c r="G23" s="4" t="n">
+      <c r="G23" s="12" t="n">
         <v>403</v>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="12" t="inlineStr">
         <is>
           <t>Forbidden</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I23" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr"/>
+      <c r="J23" s="13" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -4101,53 +4155,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr"/>
+      <c r="J24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>API-ART-12</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>/users/articles/:id</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Delete article (no auth)</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="G25" s="12" t="n">
         <v>401</v>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H25" s="12" t="inlineStr">
         <is>
           <t>Unauthorized</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I25" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr"/>
+      <c r="J25" s="13" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -4193,7 +4247,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr"/>
+      <c r="J26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -4239,7 +4293,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr"/>
+      <c r="J27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -4285,7 +4339,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J28" s="3" t="inlineStr"/>
+      <c r="J28" s="11" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -4331,7 +4385,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr"/>
+      <c r="J29" s="11" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -4377,53 +4431,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr"/>
+      <c r="J30" s="11" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>API-ART-18</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>/users/articles/:id/comments</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Add comment (empty)</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="12" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="G31" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H31" s="12" t="inlineStr">
         <is>
           <t>Content required</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I31" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr"/>
+      <c r="J31" s="13" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -4469,53 +4523,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr"/>
+      <c r="J32" s="11" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>API-ART-20</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="12" t="inlineStr">
         <is>
           <t>/users/articles/comments/:id</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Delete others comment</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G33" s="4" t="n">
+      <c r="G33" s="12" t="n">
         <v>403</v>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H33" s="12" t="inlineStr">
         <is>
           <t>Forbidden</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I33" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr"/>
+      <c r="J33" s="13" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -4561,7 +4615,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J34" s="3" t="inlineStr"/>
+      <c r="J34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -4607,7 +4661,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr"/>
+      <c r="J35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -4653,53 +4707,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J36" s="3" t="inlineStr"/>
+      <c r="J36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>API-TM-04</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>/users/matchmaking/lobbies</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Get all lobbies (no auth)</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F37" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G37" s="4" t="n">
+      <c r="G37" s="12" t="n">
         <v>401</v>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="H37" s="12" t="inlineStr">
         <is>
           <t>Unauthorized</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="I37" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr"/>
+      <c r="J37" s="13" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -4745,7 +4799,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J38" s="3" t="inlineStr"/>
+      <c r="J38" s="11" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -4791,7 +4845,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J39" s="3" t="inlineStr"/>
+      <c r="J39" s="11" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -4837,53 +4891,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J40" s="3" t="inlineStr"/>
+      <c r="J40" s="11" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>API-TM-08</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B41" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>/users/matchmaking/lobbies/:id</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Lobby detail (invalid)</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F41" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G41" s="4" t="n">
+      <c r="G41" s="12" t="n">
         <v>404</v>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="H41" s="12" t="inlineStr">
         <is>
           <t>Not found</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I41" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr"/>
+      <c r="J41" s="13" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -4929,99 +4983,99 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J42" s="3" t="inlineStr"/>
+      <c r="J42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>API-TM-10</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr">
         <is>
           <t>/users/matchmaking/lobbies</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D43" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Create lobby (no name)</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="F43" s="12" t="inlineStr">
         <is>
           <t>{"competition_id":1}</t>
         </is>
       </c>
-      <c r="G43" s="4" t="n">
+      <c r="G43" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="H43" s="12" t="inlineStr">
         <is>
           <t>Name required</t>
         </is>
       </c>
-      <c r="I43" s="4" t="inlineStr">
+      <c r="I43" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J43" s="4" t="inlineStr"/>
+      <c r="J43" s="13" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>API-TM-11</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C44" s="12" t="inlineStr">
         <is>
           <t>/users/matchmaking/lobbies</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D44" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" s="12" t="inlineStr">
         <is>
           <t>Create lobby (no auth)</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F44" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G44" s="4" t="n">
+      <c r="G44" s="12" t="n">
         <v>401</v>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="H44" s="12" t="inlineStr">
         <is>
           <t>Unauthorized</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="I44" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J44" s="4" t="inlineStr"/>
+      <c r="J44" s="13" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -5067,53 +5121,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J45" s="3" t="inlineStr"/>
+      <c r="J45" s="11" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>API-TM-13</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C46" s="12" t="inlineStr">
         <is>
           <t>/users/matchmaking/lobbies/:id</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D46" s="12" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E46" s="12" t="inlineStr">
         <is>
           <t>Delete others lobby</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F46" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G46" s="4" t="n">
+      <c r="G46" s="12" t="n">
         <v>403</v>
       </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="H46" s="12" t="inlineStr">
         <is>
           <t>Forbidden</t>
         </is>
       </c>
-      <c r="I46" s="4" t="inlineStr">
+      <c r="I46" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J46" s="4" t="inlineStr"/>
+      <c r="J46" s="13" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -5159,53 +5213,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J47" s="3" t="inlineStr"/>
+      <c r="J47" s="11" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A48" s="12" t="inlineStr">
         <is>
           <t>API-TM-15</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" s="12" t="inlineStr">
         <is>
           <t>/users/matchmaking/lobbies/:id/apply</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D48" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E48" s="12" t="inlineStr">
         <is>
           <t>Apply twice</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="F48" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G48" s="4" t="n">
+      <c r="G48" s="12" t="n">
         <v>409</v>
       </c>
-      <c r="H48" s="4" t="inlineStr">
+      <c r="H48" s="12" t="inlineStr">
         <is>
           <t>Already applied/member</t>
         </is>
       </c>
-      <c r="I48" s="4" t="inlineStr">
+      <c r="I48" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J48" s="4" t="inlineStr"/>
+      <c r="J48" s="13" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -5251,7 +5305,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J49" s="3" t="inlineStr"/>
+      <c r="J49" s="11" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -5297,53 +5351,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J50" s="3" t="inlineStr"/>
+      <c r="J50" s="11" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t>API-TM-18</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>/users/matchmaking/lobbies/:id/applications/:appId</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Review without owner role</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="F51" s="12" t="inlineStr">
         <is>
           <t>{"action":"approve"}</t>
         </is>
       </c>
-      <c r="G51" s="4" t="n">
+      <c r="G51" s="12" t="n">
         <v>403</v>
       </c>
-      <c r="H51" s="4" t="inlineStr">
+      <c r="H51" s="12" t="inlineStr">
         <is>
           <t>Forbidden</t>
         </is>
       </c>
-      <c r="I51" s="4" t="inlineStr">
+      <c r="I51" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J51" s="4" t="inlineStr"/>
+      <c r="J51" s="13" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -5389,7 +5443,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J52" s="3" t="inlineStr"/>
+      <c r="J52" s="11" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -5435,53 +5489,53 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr"/>
+      <c r="J53" s="11" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="A54" s="12" t="inlineStr">
         <is>
           <t>API-TM-21</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B54" s="12" t="inlineStr">
         <is>
           <t>Team Matchmaking</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C54" s="12" t="inlineStr">
         <is>
           <t>/users/matchmaking/lobbies/:id/members/:userId</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="E54" s="12" t="inlineStr">
         <is>
           <t>Kick member (not owner)</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="F54" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G54" s="4" t="n">
+      <c r="G54" s="12" t="n">
         <v>403</v>
       </c>
-      <c r="H54" s="4" t="inlineStr">
+      <c r="H54" s="12" t="inlineStr">
         <is>
           <t>Forbidden</t>
         </is>
       </c>
-      <c r="I54" s="4" t="inlineStr">
+      <c r="I54" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J54" s="4" t="inlineStr"/>
+      <c r="J54" s="13" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -5527,7 +5581,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr"/>
+      <c r="J55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -5573,7 +5627,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J56" s="3" t="inlineStr"/>
+      <c r="J56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -5619,7 +5673,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J57" s="3" t="inlineStr"/>
+      <c r="J57" s="11" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -5665,7 +5719,7 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J58" s="3" t="inlineStr"/>
+      <c r="J58" s="11" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -5711,99 +5765,99 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J59" s="3" t="inlineStr"/>
+      <c r="J59" s="11" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+      <c r="A60" s="12" t="inlineStr">
         <is>
           <t>API-SF-03</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>Selection Form</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C60" s="12" t="inlineStr">
         <is>
           <t>/operational/add-competitions</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D60" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="E60" s="12" t="inlineStr">
         <is>
           <t>Add competition (no auth)</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="F60" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G60" s="4" t="n">
+      <c r="G60" s="12" t="n">
         <v>401</v>
       </c>
-      <c r="H60" s="4" t="inlineStr">
+      <c r="H60" s="12" t="inlineStr">
         <is>
           <t>Unauthorized</t>
         </is>
       </c>
-      <c r="I60" s="4" t="inlineStr">
+      <c r="I60" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J60" s="4" t="inlineStr"/>
+      <c r="J60" s="13" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
+      <c r="A61" s="12" t="inlineStr">
         <is>
           <t>API-SF-04</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>Selection Form</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C61" s="12" t="inlineStr">
         <is>
           <t>/operational/add-competitions</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="E61" s="12" t="inlineStr">
         <is>
           <t>Add with empty questions when enabled</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr">
+      <c r="F61" s="12" t="inlineStr">
         <is>
           <t>{"name":"Comp","selection_enabled":true,"questions":[]}</t>
         </is>
       </c>
-      <c r="G61" s="4" t="n">
+      <c r="G61" s="12" t="n">
         <v>422</v>
       </c>
-      <c r="H61" s="4" t="inlineStr">
+      <c r="H61" s="12" t="inlineStr">
         <is>
           <t>Validation error</t>
         </is>
       </c>
-      <c r="I61" s="4" t="inlineStr">
+      <c r="I61" s="12" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="J61" s="4" t="inlineStr"/>
+      <c r="J61" s="13" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -5849,10 +5903,10 @@
           <t>Positive</t>
         </is>
       </c>
-      <c r="J62" s="3" t="inlineStr"/>
+      <c r="J62" s="11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:J62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>